<commit_message>
feat: actualizar agrupaciones para programas 4028, 4032, 4034, 4036 en seeder
</commit_message>
<xml_diff>
--- a/files_tests/FORMATO DE CARGA - ADM. DE EMPRESAS (D).xlsx
+++ b/files_tests/FORMATO DE CARGA - ADM. DE EMPRESAS (D).xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\OneDrive\Escritorio\Proyecto_Mallas\mallas\files_tests\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Debian\home\sergio\mallas\Proyecto-Mallas\files_tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12E280F6-E4E2-4CFB-B573-3ADDABD0C108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B3B475A-6A87-4616-898F-06BEB53E1B68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1842,7 +1842,7 @@
         <v>1000044</v>
       </c>
       <c r="E56" s="18" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F56" s="19"/>
       <c r="G56" s="20"/>

</xml_diff>